<commit_message>
Canevas : ajout du logiciel « AD » (colonne Oui/Non) et fiabilisation du test d'intégration
Logiciel « AD » figé comme 6e logiciel des ordinateurs, groupé après « Sysbudget » :
- Modèle canevas-vierge.xlsx : nouvelle colonne « AD » (M), liste Oui/Non étendue à H:M,
  validation statut décalée en Q ; mise en forme conditionnelle et autres validations préservées.
- DTO LigneOrdinateur (champ ad), lecteur (AD en 12, RAM→Observations décalés +1, sonde 18),
  écrivain (pré-remplissage AD + mefcStatut 16/17), intégration (logicielsDe), consolidation (sigOrd).
- Migration V14 : semis idempotent du logiciel « AD ».

Test d'intégration : le canevas d'exemple était obsolète (saisisseur non membre, aucun statut
sur les matériels) et faisait échouer ImportIntegrationTest en CI. Mise à jour du fixture
(saisisseur = membre, statut « En service » partout, colonne AD) + nouveau test local
CanevasFixtureTest qui vérifie la lecture d'AD et l'intégrabilité du canevas sans Docker.
</commit_message>
<xml_diff>
--- a/src/test/resources/canevas-exemple-rempli.xlsx
+++ b/src/test/resources/canevas-exemple-rempli.xlsx
@@ -750,6 +750,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -890,7 +891,7 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>IN001</t>
+          <t>IN002</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1373,7 +1374,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L41"/>
+  <dimension ref="A1:R41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1451,6 +1452,36 @@
           <t>Sysbudget</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>AD</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>RAM</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Processeur</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Disque dur</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Statut</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Observations</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="11" t="n"/>
@@ -1505,6 +1536,16 @@
           <t>Oui</t>
         </is>
       </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>En service</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="11" t="n"/>
@@ -1557,6 +1598,16 @@
       <c r="L3" s="11" t="inlineStr">
         <is>
           <t>Non</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>En service</t>
         </is>
       </c>
     </row>
@@ -2114,7 +2165,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2156,6 +2207,11 @@
           <t>IP</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Statut</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="11" t="n"/>
@@ -2178,6 +2234,11 @@
       <c r="F2" s="11" t="inlineStr">
         <is>
           <t>192.168.1.10</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>En service</t>
         </is>
       </c>
     </row>
@@ -2504,7 +2565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2546,6 +2607,11 @@
           <t>IP</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Statut</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="11" t="n"/>
@@ -2572,6 +2638,11 @@
       <c r="F2" s="11" t="inlineStr">
         <is>
           <t>192.168.1.2</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>En service</t>
         </is>
       </c>
     </row>
@@ -2903,7 +2974,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2933,6 +3004,11 @@
           <t>Modèle</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Statut</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="11" t="n"/>
@@ -2949,6 +3025,11 @@
       <c r="D2" s="11" t="inlineStr">
         <is>
           <t>Vision</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>En service</t>
         </is>
       </c>
     </row>

</xml_diff>